<commit_message>
Confirm OLSSR17 solid state relay price at $650
Sheffield confirmed $650, matching the 76-100A single-phase band the
mapping already used, so the row is no longer flagged for review. The
three-phase SKU draws on the same confirmed band.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XxJvecb9EHw919ig8p38oT
</commit_message>
<xml_diff>
--- a/olympic-new-compare-audit.xlsx
+++ b/olympic-new-compare-audit.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1196" uniqueCount="901">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1196" uniqueCount="902">
   <si>
     <t xml:space="preserve">SKU</t>
   </si>
@@ -2531,7 +2531,7 @@
     <t xml:space="preserve">Solid State Relays: 76-100 Amps, 1 phase</t>
   </si>
   <si>
-    <t xml:space="preserve">relays are priced by amperage; FL17/FL20/FL24 all draw 70-98A, so the 76-100A band applies</t>
+    <t xml:space="preserve">$650 confirmed by Sheffield Pottery — relays are priced by amperage and FL17/FL20/FL24 all draw 70-98A</t>
   </si>
   <si>
     <t xml:space="preserve">OLSSR173P</t>
@@ -2544,6 +2544,9 @@
   </si>
   <si>
     <t xml:space="preserve">Solid State Relays: 76-100 Amps, 3 phase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">same 76-100A band as OLSSR17, which Sheffield confirmed at $650</t>
   </si>
   <si>
     <t xml:space="preserve">OLFL20FK</t>
@@ -8912,71 +8915,71 @@
         <v/>
       </c>
     </row>
-    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A213" s="6" t="s">
+    <row r="213" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A213" s="2" t="s">
         <v>831</v>
       </c>
-      <c r="B213" s="7" t="s">
+      <c r="B213" s="3" t="s">
         <v>832</v>
       </c>
-      <c r="C213" s="8" t="s">
+      <c r="C213" s="4" t="s">
         <v>833</v>
       </c>
-      <c r="D213" s="8"/>
-      <c r="E213" s="8" t="n">
+      <c r="D213" s="4"/>
+      <c r="E213" s="4" t="n">
         <v>650</v>
       </c>
-      <c r="F213" s="7" t="s">
+      <c r="F213" s="3" t="s">
         <v>834</v>
       </c>
-      <c r="G213" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H213" s="7" t="s">
+      <c r="G213" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H213" s="3" t="s">
         <v>835</v>
       </c>
-      <c r="I213" s="9" t="str">
+      <c r="I213" s="5" t="str">
         <f aca="false">IF(OR(E213="",D213=""),"",E213/D213-1)</f>
         <v/>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A214" s="6" t="s">
+      <c r="A214" s="2" t="s">
         <v>836</v>
       </c>
-      <c r="B214" s="7" t="s">
+      <c r="B214" s="3" t="s">
         <v>837</v>
       </c>
-      <c r="C214" s="8" t="s">
+      <c r="C214" s="4" t="s">
         <v>838</v>
       </c>
-      <c r="D214" s="8"/>
-      <c r="E214" s="8" t="n">
+      <c r="D214" s="4"/>
+      <c r="E214" s="4" t="n">
         <v>925</v>
       </c>
-      <c r="F214" s="7" t="s">
+      <c r="F214" s="3" t="s">
         <v>839</v>
       </c>
-      <c r="G214" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H214" s="7" t="s">
-        <v>835</v>
-      </c>
-      <c r="I214" s="9" t="str">
+      <c r="G214" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H214" s="3" t="s">
+        <v>840</v>
+      </c>
+      <c r="I214" s="5" t="str">
         <f aca="false">IF(OR(E214="",D214=""),"",E214/D214-1)</f>
         <v/>
       </c>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="2" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="B215" s="3" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="C215" s="4" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="D215" s="4" t="n">
         <v>1158</v>
@@ -8985,7 +8988,7 @@
         <v>1235</v>
       </c>
       <c r="F215" s="3" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="G215" s="2" t="s">
         <v>13</v>
@@ -8998,10 +9001,10 @@
     </row>
     <row r="216" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="2" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="B216" s="3" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="C216" s="4" t="s">
         <v>829</v>
@@ -9026,10 +9029,10 @@
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="2" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="B217" s="3" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="C217" s="4" t="s">
         <v>28</v>
@@ -9039,7 +9042,7 @@
         <v>550</v>
       </c>
       <c r="F217" s="3" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="G217" s="2" t="s">
         <v>13</v>
@@ -9052,13 +9055,13 @@
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="2" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="B218" s="3" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="C218" s="4" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="D218" s="4" t="n">
         <v>527</v>
@@ -9067,7 +9070,7 @@
         <v>530</v>
       </c>
       <c r="F218" s="3" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="G218" s="2" t="s">
         <v>13</v>
@@ -9080,10 +9083,10 @@
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="2" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="B219" s="3" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="C219" s="4" t="s">
         <v>47</v>
@@ -9095,7 +9098,7 @@
         <v>545</v>
       </c>
       <c r="F219" s="3" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="G219" s="2" t="s">
         <v>13</v>
@@ -9108,13 +9111,13 @@
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="2" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="B220" s="3" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="C220" s="4" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="D220" s="4" t="n">
         <v>942</v>
@@ -9123,7 +9126,7 @@
         <v>1195</v>
       </c>
       <c r="F220" s="3" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="G220" s="2" t="s">
         <v>13</v>
@@ -9136,13 +9139,13 @@
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="2" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="B221" s="3" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="C221" s="4" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="D221" s="4" t="n">
         <v>2143</v>
@@ -9151,7 +9154,7 @@
         <v>2190</v>
       </c>
       <c r="F221" s="3" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="G221" s="2" t="s">
         <v>13</v>
@@ -9164,13 +9167,13 @@
     </row>
     <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="2" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="B222" s="3" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="C222" s="4" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="D222" s="4" t="n">
         <v>2143</v>
@@ -9179,7 +9182,7 @@
         <v>2270</v>
       </c>
       <c r="F222" s="3" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="G222" s="2" t="s">
         <v>13</v>
@@ -9192,13 +9195,13 @@
     </row>
     <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="2" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="B223" s="3" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="C223" s="4" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="D223" s="4" t="n">
         <v>2223</v>
@@ -9207,7 +9210,7 @@
         <v>2270</v>
       </c>
       <c r="F223" s="3" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="G223" s="2" t="s">
         <v>13</v>
@@ -9220,10 +9223,10 @@
     </row>
     <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="2" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="B224" s="3" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="C224" s="4" t="s">
         <v>106</v>
@@ -9235,7 +9238,7 @@
         <v>3510</v>
       </c>
       <c r="F224" s="3" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="G224" s="2" t="s">
         <v>13</v>
@@ -9248,13 +9251,13 @@
     </row>
     <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="2" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="B225" s="3" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="C225" s="4" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="D225" s="4" t="n">
         <v>4256</v>
@@ -9263,7 +9266,7 @@
         <v>4680</v>
       </c>
       <c r="F225" s="3" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="G225" s="2" t="s">
         <v>13</v>
@@ -9276,13 +9279,13 @@
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="2" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="B226" s="3" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="C226" s="4" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="D226" s="4" t="n">
         <v>2575</v>
@@ -9291,7 +9294,7 @@
         <v>2830</v>
       </c>
       <c r="F226" s="3" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="G226" s="2" t="s">
         <v>13</v>
@@ -9304,13 +9307,13 @@
     </row>
     <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="2" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="B227" s="3" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="C227" s="4" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="D227" s="4" t="n">
         <v>9755</v>
@@ -9319,7 +9322,7 @@
         <v>10750</v>
       </c>
       <c r="F227" s="3" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="G227" s="2" t="s">
         <v>13</v>
@@ -9332,13 +9335,13 @@
     </row>
     <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="2" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="B228" s="3" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="C228" s="4" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="D228" s="4" t="n">
         <v>6680</v>
@@ -9347,7 +9350,7 @@
         <v>7500</v>
       </c>
       <c r="F228" s="3" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="G228" s="2" t="s">
         <v>13</v>
@@ -9360,13 +9363,13 @@
     </row>
     <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="2" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="B229" s="3" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="C229" s="4" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="D229" s="4" t="n">
         <v>16635</v>
@@ -9381,7 +9384,7 @@
         <v>13</v>
       </c>
       <c r="H229" s="3" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="I229" s="5" t="n">
         <f aca="false">IF(OR(E229="",D229=""),"",E229/D229-1)</f>
@@ -9390,13 +9393,13 @@
     </row>
     <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="2" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="B230" s="3" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="C230" s="4" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="D230" s="4" t="n">
         <v>24735</v>
@@ -9405,7 +9408,7 @@
         <v>27250</v>
       </c>
       <c r="F230" s="3" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="G230" s="2" t="s">
         <v>13</v>
@@ -9418,10 +9421,10 @@
     </row>
     <row r="231" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="2" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="B231" s="3" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="C231" s="4" t="s">
         <v>678</v>
@@ -9439,7 +9442,7 @@
         <v>24</v>
       </c>
       <c r="H231" s="3" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="I231" s="5" t="n">
         <f aca="false">IF(OR(E231="",D231=""),"",E231/D231-1)</f>

</xml_diff>

<commit_message>
Confirm OL2018BR blank ring price at $480
Sheffield confirmed $480, matching the 20/20H" blank ring the mapping
already used, so the row is no longer flagged for review.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XxJvecb9EHw919ig8p38oT
</commit_message>
<xml_diff>
--- a/olympic-new-compare-audit.xlsx
+++ b/olympic-new-compare-audit.xlsx
@@ -1784,7 +1784,7 @@
     <t xml:space="preserve">Olympic: ADD a 4.5" blank ring: ADDs 1.98 cu ft.</t>
   </si>
   <si>
-    <t xml:space="preserve">SKU says 2018 but "adds 1.98 cu ft" reads like a 25" oval ring</t>
+    <t xml:space="preserve">$480 confirmed by Sheffield Pottery (20" oval ring), despite the "1.98 cu ft" in the listing</t>
   </si>
   <si>
     <t xml:space="preserve">OL25HOFK</t>
@@ -7120,29 +7120,29 @@
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A145" s="6" t="s">
+      <c r="A145" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="B145" s="7" t="s">
+      <c r="B145" s="3" t="s">
         <v>585</v>
       </c>
-      <c r="C145" s="8" t="s">
+      <c r="C145" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D145" s="8"/>
-      <c r="E145" s="8" t="n">
+      <c r="D145" s="4"/>
+      <c r="E145" s="4" t="n">
         <v>480</v>
       </c>
-      <c r="F145" s="7" t="s">
+      <c r="F145" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G145" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H145" s="7" t="s">
+      <c r="G145" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H145" s="3" t="s">
         <v>586</v>
       </c>
-      <c r="I145" s="9" t="str">
+      <c r="I145" s="5" t="str">
         <f aca="false">IF(OR(E145="",D145=""),"",E145/D145-1)</f>
         <v/>
       </c>

</xml_diff>